<commit_message>
Monthly data update for Wed 07/16/2025
</commit_message>
<xml_diff>
--- a/raw_data/aaa/Monthly AAA.xlsx
+++ b/raw_data/aaa/Monthly AAA.xlsx
@@ -754,13 +754,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1025,7 +1018,7 @@
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="10.9090909090909" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5454545454545" style="2" customWidth="1"/>
+    <col min="2" max="2" width="8.81818181818182" style="2" customWidth="1"/>
     <col min="3" max="3" width="14.1818181818182" style="3" customWidth="1"/>
     <col min="5" max="5" width="10.0909090909091" customWidth="1"/>
   </cols>
@@ -1049,7 +1042,7 @@
         <v>45658</v>
       </c>
       <c r="C2" s="6">
-        <v>15730</v>
+        <v>74911</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1060,7 +1053,7 @@
         <v>45713</v>
       </c>
       <c r="C3" s="6">
-        <v>15265</v>
+        <v>75481</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1071,7 +1064,7 @@
         <v>45741</v>
       </c>
       <c r="C4" s="6">
-        <v>15111</v>
+        <v>75976</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1082,7 +1075,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="6">
-        <v>14710</v>
+        <v>76356</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1093,7 +1086,7 @@
         <v>45802</v>
       </c>
       <c r="C6" s="6">
-        <v>15438</v>
+        <v>77062</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1104,7 +1097,7 @@
         <v>45833</v>
       </c>
       <c r="C7" s="6">
-        <v>14934</v>
+        <v>77735</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1115,7 +1108,7 @@
         <v>45658</v>
       </c>
       <c r="C8" s="6">
-        <v>9082</v>
+        <v>78777</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1126,7 +1119,7 @@
         <v>45713</v>
       </c>
       <c r="C9" s="6">
-        <v>8902</v>
+        <v>79308</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1137,7 +1130,7 @@
         <v>45741</v>
       </c>
       <c r="C10" s="6">
-        <v>8841</v>
+        <v>79778</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1148,7 +1141,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="6">
-        <v>8879</v>
+        <v>80313</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1159,7 +1152,7 @@
         <v>45802</v>
       </c>
       <c r="C12" s="6">
-        <v>8923</v>
+        <v>80851</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1170,7 +1163,7 @@
         <v>45833</v>
       </c>
       <c r="C13" s="6">
-        <v>8598</v>
+        <v>81294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monthly data update for Wed 07/30/2025
</commit_message>
<xml_diff>
--- a/raw_data/aaa/Monthly AAA.xlsx
+++ b/raw_data/aaa/Monthly AAA.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="6">
   <si>
     <t>AAA Location</t>
   </si>
@@ -1014,7 +1014,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="10.9090909090909" style="1" customWidth="1"/>
@@ -1102,13 +1102,13 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B8" s="5">
-        <v>45658</v>
+        <v>45863</v>
       </c>
       <c r="C8" s="6">
-        <v>78777</v>
+        <v>77988</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1116,10 +1116,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="5">
-        <v>45713</v>
+        <v>45658</v>
       </c>
       <c r="C9" s="6">
-        <v>79308</v>
+        <v>78777</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1127,32 +1127,32 @@
         <v>5</v>
       </c>
       <c r="B10" s="5">
-        <v>45741</v>
+        <v>45713</v>
       </c>
       <c r="C10" s="6">
-        <v>79778</v>
+        <v>79308</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>4</v>
+      <c r="B11" s="5">
+        <v>45741</v>
       </c>
       <c r="C11" s="6">
-        <v>80313</v>
+        <v>79778</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="5">
-        <v>45802</v>
+      <c r="B12" s="5" t="s">
+        <v>4</v>
       </c>
       <c r="C12" s="6">
-        <v>80851</v>
+        <v>80313</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1160,10 +1160,32 @@
         <v>5</v>
       </c>
       <c r="B13" s="5">
+        <v>45802</v>
+      </c>
+      <c r="C13" s="6">
+        <v>80851</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="5">
         <v>45833</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C14" s="6">
         <v>81294</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" spans="1:3">
+      <c r="A15" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="5">
+        <v>45863</v>
+      </c>
+      <c r="C15" s="6">
+        <v>81517</v>
       </c>
     </row>
   </sheetData>

</xml_diff>